<commit_message>
Auto update Pengadaan 2026-09-02 08:09:06
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-02).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-09-02).xlsx
@@ -3732,10 +3732,10 @@
         <v>962557890</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>705820440</v>
+        <v>962557890</v>
       </c>
       <c r="K19" s="7" t="inlineStr">
         <is>
@@ -6426,10 +6426,10 @@
         <v>60673958430.41</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>28305839637</v>
+        <v>28562577087</v>
       </c>
       <c r="K67" s="12" t="n">
         <v>7</v>
@@ -10202,13 +10202,13 @@
         <v>5</v>
       </c>
       <c r="H65" s="6" t="n">
-        <v>1559826000</v>
+        <v>2247425999.97</v>
       </c>
       <c r="I65" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J65" s="6" t="n">
-        <v>1559826000</v>
+        <v>2247425999.97</v>
       </c>
       <c r="K65" s="7" t="inlineStr">
         <is>
@@ -10300,13 +10300,13 @@
         <v>151</v>
       </c>
       <c r="H67" s="13" t="n">
-        <v>64567432791.01</v>
+        <v>65255032790.98</v>
       </c>
       <c r="I67" s="12" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J67" s="13" t="n">
-        <v>60508498991</v>
+        <v>61196098990.97</v>
       </c>
       <c r="K67" s="12" t="n">
         <v>29</v>

</xml_diff>